<commit_message>
- Corrected toBeWasted field in excel files - Rounding the Projected Stock Waste field
</commit_message>
<xml_diff>
--- a/api/templates/export/supplies-by-lot/en.xlsx
+++ b/api/templates/export/supplies-by-lot/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\supplies\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\export\supplies-by-lot\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E20541C-4A55-450C-AFEA-1606A8038566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplies" sheetId="1" r:id="rId1"/>
@@ -147,9 +148,6 @@
     <t>&lt;expiresOn&gt;</t>
   </si>
   <si>
-    <t>&lt;expires&gt;</t>
-  </si>
-  <si>
     <t>Aspect Supplies</t>
   </si>
   <si>
@@ -162,13 +160,16 @@
     <t>Printed on &lt;date&gt;</t>
   </si>
   <si>
-    <t># Expires</t>
+    <t>Lot Number</t>
+  </si>
+  <si>
+    <t>&lt;lotNumber&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
@@ -176,7 +177,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -184,7 +185,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -192,7 +193,7 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -200,7 +201,7 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -208,7 +209,7 @@
       <u/>
       <sz val="12"/>
       <color theme="11"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -331,48 +332,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -400,7 +401,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -737,43 +738,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.5" style="4" customWidth="1"/>
-    <col min="2" max="2" width="31.125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="32.44140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" style="2" customWidth="1"/>
     <col min="3" max="3" width="22" style="2" customWidth="1"/>
-    <col min="4" max="4" width="21.625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="19.375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="5" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="5" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>33</v>
       </c>
@@ -784,15 +785,15 @@
         <v>35</v>
       </c>
       <c r="D5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>37</v>
@@ -801,10 +802,10 @@
         <v>38</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>39</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -819,13 +820,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.21875" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -839,7 +840,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -850,7 +851,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -861,7 +862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -872,7 +873,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -883,7 +884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -894,7 +895,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -905,7 +906,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -916,7 +917,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -927,7 +928,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -938,7 +939,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -949,7 +950,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -960,7 +961,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -971,7 +972,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -982,7 +983,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -993,7 +994,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1004,7 +1005,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1015,7 +1016,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1026,7 +1027,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1037,7 +1038,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1048,7 +1049,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1059,7 +1060,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1070,7 +1071,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1081,7 +1082,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1092,7 +1093,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1103,7 +1104,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1114,7 +1115,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>